<commit_message>
Release v1.1.1: clarify teaching and improve reading workflows
</commit_message>
<xml_diff>
--- a/文献下载清单.xlsx
+++ b/文献下载清单.xlsx
@@ -7348,10 +7348,8 @@
           <t>Jöreskog, K. G.</t>
         </is>
       </c>
-      <c r="E81" s="2" t="inlineStr">
-        <is>
-          <t>1973</t>
-        </is>
+      <c r="E81" s="2" t="n">
+        <v>1970</v>
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
@@ -7380,7 +7378,7 @@
       </c>
       <c r="K81" s="2" t="inlineStr">
         <is>
-          <t>LISREL 的理论奠基</t>
+          <t>线性结构方程系统的早期报告；此DOI对应1970年ETS报告。</t>
         </is>
       </c>
       <c r="L81" s="2" t="inlineStr">

</xml_diff>